<commit_message>
chore: update FIFA World Cup 2026 data
</commit_message>
<xml_diff>
--- a/fifa/fifa_data.xlsx
+++ b/fifa/fifa_data.xlsx
@@ -2587,7 +2587,11 @@
           <t>Should Bellingham have been sent off vs. Ghana?</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>The headline questions whether Bellingham should have received a red card during a FIFA World Cup 2026 match against Ghana. This prompts discussion regarding the referee's decision and its potential implications.</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>https://a.espncdn.com/media/motion/2026/0624/dm_260624_COM_SOC_ANALYSIS_Should_Bellingham_have_been_sent_off_vs_Ghana_2026_6_24/dm_260624_COM_SOC_ANALYSIS_Should_Bellingham_have_been_sent_off_vs_Ghana_2026_6_24.jpg</t>
@@ -2679,7 +2683,11 @@
           <t>Did Mendes' free kick reveal a different side to Ronaldo?</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>A FIFA World Cup 2026 headline questions if a free kick taken by Mendes revealed an unexpected aspect of Cristiano Ronaldo's personality or role. It suggests the article will analyze Ronaldo's reaction to the event, exploring what it signifies about his evolving leadership or presence within the team.</t>
+        </is>
+      </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>https://a.espncdn.com/media/motion/2026/0624/dm_260624_COM_SOC_ANALYSIS_Did_Mendes_free_kick_reveal_a_different_side_to_Ronaldo_2026_6_24/dm_260624_COM_SOC_ANALYSIS_Did_Mendes_free_kick_reveal_a_different_side_to_Ronaldo_2026_6_24.jpg</t>

</xml_diff>